<commit_message>
Rewrite Sugar News 2026-09-03 summaries
</commit_message>
<xml_diff>
--- a/reports/2026/09/Sugar News 2026-09-03.xlsx
+++ b/reports/2026/09/Sugar News 2026-09-03.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="55" customWidth="1" style="2" min="2" max="2"/>
@@ -505,7 +505,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="146.65" customHeight="1" s="2">
+    <row r="2" ht="180" customHeight="1" s="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
           <t>印度</t>
@@ -513,63 +513,46 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>印度零售市场显示零售糖价，糖价变动幅度为3.85%。印度零售糖价仅披露当前水平，缺少前期比较时不单独改变供需方向判断。来源：hindustantimes.com（https://www.hindustantimes.com/india-news/retail-sugar-price-drops-3-85-percent-to-rs-62-57-kg-in-a-week-govt-data-101788454755161.html）。影响：中性</t>
+          <t>印度消费者事务部数据显示，全国平均零售糖价一周下跌3.85%至62.57卢比/公斤，低于一周前65.08卢比/公斤；9月2日平均批发价由一周前60.39卢比/公斤降至57.62卢比/公斤，但零售价仍比一个月前49.33卢比/公斤高27%。价格回落发生在印度政府允许进口100万吨食糖、收紧大用户和经销商库存限制之后，进口和限库增加可流通糖源、压低囤货与节前补库溢价，短期利空印度现货糖价。政府同时把2025/26营销年产量预估从3430万吨下调至3060万吨、年需求为2800万-2850万吨，说明中期供应缓冲仍有限。来源：The Times of India（https://timesofindia.indiatimes.com/business/india-business/sugar-prices-ease-retail-rates-fall-3-85-to-rs-62-57/kg-in-a-week/articleshow/133733317.cms）。影响：利空糖价</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>中性：印度零售糖价仅披露当前水平，缺少前期比较时不单独改变供需方向判断。</t>
+          <t>利空：印度政府允许进口100万吨食糖并收紧库存限制后，零售和批发糖价周度回落，进口糖源和限库措施压低囤货需求与节前补库溢价，短期利空印度现货糖价。</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="156" customHeight="1" s="2">
+    <row r="3" ht="162.6" customHeight="1" s="2">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>印度</t>
+          <t>泰国</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>印度零售市场显示零售糖价，糖价下跌3.85%。印度零售糖价下跌说明当地供应压力增加或采购需求转弱，短期压制现货糖价。来源：The Times of India（https://timesofindia.indiatimes.com/business/india-business/sugar-prices-ease-retail-rates-fall-3-85-to-rs-62-57/kg-in-a-week/articleshow/133733317.cms）。影响：利空糖价</t>
+          <t>Open-Meteo 9月3日预报显示，9月4日至9月10日泰国东北部呵叻、孔敬、乌隆他尼、猜也蓬，北部那空沙旺、甘烹碧、素可泰、彭世洛，中西部北碧、华富里、素攀武里、猜纳和东部沙缴、春武里等甘蔗区有降雨，其中沙缴累计约171.7mm、甘烹碧约149.8mm、加拉信约139.9mm。泰国甘蔗处于生长期，上述降雨补充土壤水分、改善单产形成条件，提高后期甘蔗和食糖供应预期，利空糖价。来源：Open-Meteo（https://api.open-meteo.com/v1/forecast）。影响：利空糖价</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>利空：印度零售糖价下跌说明当地供应压力增加或采购需求转弱，短期压制现货糖价。</t>
+          <t>利空：泰国主产区生长期降雨补充土壤水分并改善单产形成条件，提高后期甘蔗和食糖供应预期，利空糖价。</t>
         </is>
       </c>
     </row>
     <row r="4" ht="180" customHeight="1" s="2">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>泰国</t>
+          <t>菲律宾</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Open-Meteo预报显示（2026-09-04至2026-09-10），泰国东北部（呵叻、孔敬、乌隆他尼、猜也蓬）；北部（那空沙旺、甘烹碧、素可泰、彭世洛）；中部及西部（北碧、华富里、素攀武里、猜纳）；东部（沙缴、春武里）等主要甘蔗产区存在降雨预报，实际可用预报期为7日，累计预测降雨较高的监测点包括沙缴约171.7mm、甘烹碧约149.8mm、加拉信约139.9mm。当前处于甘蔗生长阶段，降雨有利于补充土壤水分、改善墒情并促进甘蔗生长和单产形成，提高后期甘蔗及食糖产量预期。来源：Open-Meteo（https://api.open-meteo.com/v1/forecast）。影响：利空糖价</t>
+          <t>近期重要消息：菲律宾农业部和能源部正在评估将乙醇强制掺混比例由10%提高至15%，并讨论使用糖蜜、甘蔗汁、本地玉米和棕榈油等原料，同时利用闲置酒精产能。菲律宾糖基原料当前每年生产约3.25亿-3.85亿升生物乙醇，行业总产能超过5亿升；若新增掺混需求仍由糖蜜和甘蔗汁承担，将把可发酵糖源从制糖链条转向乙醇，减少可结晶糖供应并利多糖价。由于国家生物乙醇标准仍在公开咨询且政府也在评估玉米等非糖原料，非糖原料放量会削弱对食糖供应的挤压。来源：菲律宾农业部（https://www.da.gov.ph/da-doe-seek-cheaper-feedstock-to-expand-bioethanol/）。影响：利多糖价</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>利空：甘蔗生长阶段的降雨有利于补充土壤水分、改善墒情并促进甘蔗生长和单产形成，从而增加未来甘蔗及食糖供应预期，因此利空糖价。</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="149.4" customHeight="1" s="2">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>菲律宾</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>菲律宾糖业相关机构公布乙醇掺混或燃料政策，披露15%。若新增乙醇需求由B重糖蜜、糖浆或甘蔗汁满足，糖厂会把这些可发酵糖源送入乙醇装置；其中B重糖蜜、糖浆和甘蔗汁会减少可结晶成白糖的蔗糖量。来源：BioEnergy Times（https://bioenergytimes.com/philippines-considers-raising-ethanol-blend-to-15-as-it-explores-new-feedstock/）。影响：利多糖价</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>利多：若新增乙醇需求由B重糖蜜、糖浆或甘蔗汁满足，糖厂会把这些可发酵糖源送入乙醇装置；其中B重糖蜜、糖浆和甘蔗汁会减少可结晶成白糖的蔗糖量，从而减少食糖供应预期并支撑糖价。</t>
+          <t>利多：菲律宾若把乙醇掺混比例从10%提高至15%，且新增需求继续由糖蜜和甘蔗汁承担，会分流制糖糖源、减少可结晶糖供应；玉米等非糖原料放量会削弱这一利多。</t>
         </is>
       </c>
     </row>

</xml_diff>